<commit_message>
Extraer datos de la base de datos, y añadir el campo de nombre excel en el back
</commit_message>
<xml_diff>
--- a/app_horarios/datos/excel/export-14-04.xlsx
+++ b/app_horarios/datos/excel/export-14-04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Desktop\Ingeniería informática\4º Trabajo de Fin de Grado\Trabajo-Fin-de-Grado-2025-2026\app_horarios\datos\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA71B4B-D734-42F7-A5AA-11D7E5538F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD2AB3E-3D29-476B-8CE6-3F864B1BE876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="asignaturas" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="225">
   <si>
     <t>IDASIGNATURA</t>
   </si>
@@ -697,6 +697,21 @@
   </si>
   <si>
     <t>OBSERVACIONES</t>
+  </si>
+  <si>
+    <t>Castillo</t>
+  </si>
+  <si>
+    <t>Martinez</t>
+  </si>
+  <si>
+    <t>Remacha</t>
+  </si>
+  <si>
+    <t>Bargas</t>
+  </si>
+  <si>
+    <t>Maravilla</t>
   </si>
 </sst>
 </file>
@@ -2339,6 +2354,9 @@
       <c r="B2" t="s">
         <v>200</v>
       </c>
+      <c r="C2" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -2347,6 +2365,9 @@
       <c r="B3" t="s">
         <v>201</v>
       </c>
+      <c r="C3" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -2369,6 +2390,9 @@
       <c r="B5" t="s">
         <v>202</v>
       </c>
+      <c r="C5" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -2419,6 +2443,9 @@
       <c r="B9" t="s">
         <v>210</v>
       </c>
+      <c r="C9" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -2426,6 +2453,9 @@
       </c>
       <c r="B10" t="s">
         <v>210</v>
+      </c>
+      <c r="C10" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>